<commit_message>
Add Sandisk and Nebius to the RSA source and all language tabs
Both fit the existing template without needing the ticker/short-connector
fallback (Sandisk=7 chars, Nebius=6 chars, both under the tightest
Headline 5 budget in every language), so all headlines and descriptions
render in full template form across English + the 6 translations.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WziQuJ5yimzFpKMNwdyYsQ
</commit_message>
<xml_diff>
--- a/data/reference/Stock_Campaign_RSA_Translations.xlsx
+++ b/data/reference/Stock_Campaign_RSA_Translations.xlsx
@@ -676,11 +676,6 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NVIDIA stock</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>NVDA</t>
@@ -814,11 +809,6 @@
           <t>TESLA</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>TESLA stock</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
           <t>TSLA</t>
@@ -952,11 +942,6 @@
           <t>AMD</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>AMD stock</t>
-        </is>
-      </c>
       <c r="D4" t="inlineStr">
         <is>
           <t>AMD</t>
@@ -1090,11 +1075,6 @@
           <t>ASML</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>ASML stock</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>ASML</t>
@@ -1228,11 +1208,6 @@
           <t>Intel</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Intel stock</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>INTC</t>
@@ -1366,11 +1341,6 @@
           <t>Palantir</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Palantir stock</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>PLTR</t>
@@ -1504,11 +1474,6 @@
           <t>Rheinmetall</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Rheinmetall stock</t>
-        </is>
-      </c>
       <c r="D8" t="inlineStr">
         <is>
           <t>RHM.DE</t>
@@ -1642,11 +1607,6 @@
           <t>Google</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Google stock</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
           <t>GOOG</t>
@@ -1780,11 +1740,6 @@
           <t>AMAZON</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>AMAZON stock</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>AMZN</t>
@@ -1918,11 +1873,6 @@
           <t>META</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>META stock</t>
-        </is>
-      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>META</t>
@@ -2056,11 +2006,6 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Microsoft stock</t>
-        </is>
-      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>MSFT</t>
@@ -2194,11 +2139,6 @@
           <t>Novo Nordisk</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Novo Nordisk stock</t>
-        </is>
-      </c>
       <c r="D13" t="inlineStr">
         <is>
           <t>NVO</t>
@@ -2332,11 +2272,6 @@
           <t>Gamestop</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Gamestop stock</t>
-        </is>
-      </c>
       <c r="D14" t="inlineStr">
         <is>
           <t>GME</t>
@@ -2470,11 +2405,6 @@
           <t>APPLE</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>APPLE stock</t>
-        </is>
-      </c>
       <c r="D15" t="inlineStr">
         <is>
           <t>AAPL</t>
@@ -2608,11 +2538,6 @@
           <t>Netflix</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Netflix stock</t>
-        </is>
-      </c>
       <c r="D16" t="inlineStr">
         <is>
           <t>NFLX</t>
@@ -2746,11 +2671,6 @@
           <t>Adyen</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Adyen stock</t>
-        </is>
-      </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>ADYEN.AS</t>
@@ -2884,11 +2804,6 @@
           <t>Micron</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Micron stock</t>
-        </is>
-      </c>
       <c r="D18" t="inlineStr">
         <is>
           <t>MU</t>
@@ -3022,11 +2937,6 @@
           <t>SMCI</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>SMCI stock</t>
-        </is>
-      </c>
       <c r="D19" t="inlineStr">
         <is>
           <t>SMCI</t>
@@ -3160,11 +3070,6 @@
           <t>Coinbase</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Coinbase stock</t>
-        </is>
-      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>COIN</t>
@@ -3298,11 +3203,6 @@
           <t>Shell</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Shell stock</t>
-        </is>
-      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>SHEL</t>
@@ -3436,11 +3336,6 @@
           <t>Alphabet</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Alphabet stock</t>
-        </is>
-      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>GOOG</t>
@@ -3574,11 +3469,6 @@
           <t>Nokia</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Nokia stock</t>
-        </is>
-      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>NOK</t>
@@ -3712,11 +3602,6 @@
           <t>Space X</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Space X stock</t>
-        </is>
-      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>SPCX</t>
@@ -3850,11 +3735,6 @@
           <t>Take Two</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Take Two stock</t>
-        </is>
-      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>TTWO</t>
@@ -3988,11 +3868,6 @@
           <t>LVMH</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>LVMH stock</t>
-        </is>
-      </c>
       <c r="D26" t="inlineStr">
         <is>
           <t>MC.PA</t>
@@ -4264,11 +4139,6 @@
           <t>ING Group</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>ING Group stock</t>
-        </is>
-      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>ING</t>
@@ -4402,11 +4272,6 @@
           <t>Booking</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Booking stock</t>
-        </is>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>BKNG</t>
@@ -4540,11 +4405,6 @@
           <t>Booking Holdings</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Booking Holdings stock</t>
-        </is>
-      </c>
       <c r="D30" t="inlineStr">
         <is>
           <t>BKNG</t>
@@ -4678,11 +4538,6 @@
           <t>Ferrari</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Ferrari stock</t>
-        </is>
-      </c>
       <c r="D31" t="inlineStr">
         <is>
           <t>RACE</t>
@@ -4816,11 +4671,6 @@
           <t>Volkswagen</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Volkswagen stock</t>
-        </is>
-      </c>
       <c r="D32" t="inlineStr">
         <is>
           <t>VOW3.DE</t>
@@ -4954,11 +4804,6 @@
           <t>ASR</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>ASR stock</t>
-        </is>
-      </c>
       <c r="D33" t="inlineStr">
         <is>
           <t>ASRNL.AS</t>
@@ -5092,11 +4937,6 @@
           <t>CSG</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>CSG stock</t>
-        </is>
-      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>CSGS</t>
@@ -5230,11 +5070,6 @@
           <t>KLM</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>KLM stock</t>
-        </is>
-      </c>
       <c r="D35" t="inlineStr">
         <is>
           <t>AF.PA</t>
@@ -5368,11 +5203,6 @@
           <t>Ahold</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Ahold stock</t>
-        </is>
-      </c>
       <c r="D36" t="inlineStr">
         <is>
           <t>AD.AS</t>
@@ -5506,11 +5336,6 @@
           <t>Santander</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Santander stock</t>
-        </is>
-      </c>
       <c r="D37" t="inlineStr">
         <is>
           <t>SAN</t>
@@ -5644,11 +5469,6 @@
           <t>Banco Santander</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Banco Santander stock</t>
-        </is>
-      </c>
       <c r="D38" t="inlineStr">
         <is>
           <t>SAN</t>
@@ -5780,11 +5600,6 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>Air France</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Air France stock</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -5933,7 +5748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <sheetData>
     <row r="1" ht="14.4" customHeight="1">
@@ -11395,6 +11210,280 @@
       <c r="AB39" t="inlineStr">
         <is>
           <t>air-france</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk stock</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Everyone’s an investor</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Start investing with DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Enjoy low fees</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Financial power to you</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Invest in Sandisk with DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Sandisk stock</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Invest in Sandisk shares</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Invest in Sandisk stock</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Sandisk Shares</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Sandisk Stock</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>100+ international awards</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Very low trading fees</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Invest with low costs</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3M investors trust DEGIRO</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Award-winning platform</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Investing involves risk of loss. This is not investment advice.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Start investing in Sandisk stock with low costs at DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Open your account free and access 45+ markets in 30 countries.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>See why 3M investors use our award-winning platform.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>stocks</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius stock</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Everyone’s an investor</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Start investing with DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Enjoy low fees</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Financial power to you</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Invest in Nebius with DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Nebius stock</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Invest in Nebius shares</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Invest in Nebius stock</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Nebius Shares</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Nebius Stock</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>100+ international awards</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Very low trading fees</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Invest with low costs</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3M investors trust DEGIRO</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Award-winning platform</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Investing involves risk of loss. This is not investment advice.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Start investing in Nebius stock with low costs at DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Open your account free and access 45+ markets in 30 countries.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>See why 3M investors use our award-winning platform.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>stocks</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
         </is>
       </c>
     </row>
@@ -11421,7 +11510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16802,6 +16891,280 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk acciones</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO: todos pueden invertir</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Empieza a invertir con DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO: tarifas muy bajas</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO: el poder es tuyo</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Invierte en Sandisk con DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Acciones de Sandisk</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Invierte en acciones Sandisk</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Invierte en acción Sandisk</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO: acciones Sandisk</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO: acción Sandisk</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>100+ premios internacionales</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Comisiones de trading bajas</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Invierte con costes bajos</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3M inversores ya confían</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Plataforma premiada</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Invertir implica riesgo de pérdida. Esto no es asesoramiento de inversión.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Empieza a invertir en acciones de Sandisk con costes bajos en DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Abre tu cuenta gratis y accede a 45+ mercados en 30 países.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Descubre por qué 3M inversores usan nuestra plataforma premiada.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>acciones</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius acciones</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO: todos pueden invertir</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Empieza a invertir con DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO: tarifas muy bajas</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO: el poder es tuyo</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Invierte en Nebius con DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Acciones de Nebius</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Invierte en acciones Nebius</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Invierte en acción Nebius</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO: acciones Nebius</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO: acción Nebius</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>100+ premios internacionales</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Comisiones de trading bajas</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Invierte con costes bajos</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3M inversores ya confían</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Plataforma premiada</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Invertir implica riesgo de pérdida. Esto no es asesoramiento de inversión.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Empieza a invertir en acciones de Nebius con costes bajos en DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Abre tu cuenta gratis y accede a 45+ mercados en 30 países.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Descubre por qué 3M inversores usan nuestra plataforma premiada.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>acciones</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16813,7 +17176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22194,6 +22557,280 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk Aktie</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Jeder kann investieren</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Jetzt investieren mit DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO: sehr niedrige Gebühren</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO: finanzielle Stärke</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Investiere in Sandisk - DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Sandisk Aktie</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Investiere in Sandisk-Aktien</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Investiere in Sandisk-Aktie</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Sandisk-Aktien</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO: Sandisk-Aktie</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>100+ internationale Awards</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Sehr niedrige Handelsgebühren</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Investieren zu geringen Kosten</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3 Mio. Anleger vertrauen uns</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Preisgekrönte Plattform</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Investieren ist mit Verlustrisiko verbunden. Dies ist keine Anlageberatung.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Investiere in Sandisk-Aktien zu niedrigen Kosten bei DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Eröffne dein Konto gratis und erhalte Zugang zu 45+ Märkten in 30 Ländern.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Erfahre, warum 3 Mio. Anleger unsere preisgekrönte Plattform nutzen.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>Aktien</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius Aktie</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Jeder kann investieren</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Jetzt investieren mit DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO: sehr niedrige Gebühren</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO: finanzielle Stärke</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Investiere in Nebius - DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Nebius Aktie</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Investiere in Nebius-Aktien</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Investiere in Nebius-Aktie</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Nebius-Aktien</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO: Nebius-Aktie</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>100+ internationale Awards</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Sehr niedrige Handelsgebühren</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Investieren zu geringen Kosten</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3 Mio. Anleger vertrauen uns</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Preisgekrönte Plattform</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Investieren ist mit Verlustrisiko verbunden. Dies ist keine Anlageberatung.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Investiere in Nebius-Aktien zu niedrigen Kosten bei DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Eröffne dein Konto gratis und erhalte Zugang zu 45+ Märkten in 30 Ländern.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Erfahre, warum 3 Mio. Anleger unsere preisgekrönte Plattform nutzen.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>Aktien</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -22205,7 +22842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27586,6 +28223,280 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk action</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO : chacun peut investir</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Investissez avec DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO : frais très bas</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO : le pouvoir financier</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Investir dans Sandisk - DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Action Sandisk</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Investir en actions Sandisk</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Investir dans l'action Sandisk</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO : actions Sandisk</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO : action Sandisk</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>Plus de 100 récompenses</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Frais de trading très bas</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Investissez à faible coût</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3M investisseurs satisfaits</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Plateforme primée</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Investir comporte un risque de perte. Ceci n'est pas un conseil en investissement.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Investissez dans l'action Sandisk à faible coût avec DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Ouvrez un compte gratuit et accédez à 45+ marchés dans 30 pays.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Découvrez pourquoi 3M d'investisseurs utilisent notre plateforme primée.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius action</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO : chacun peut investir</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Investissez avec DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO : frais très bas</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO : le pouvoir financier</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Investir dans Nebius - DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Action Nebius</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Investir en actions Nebius</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Investir dans l'action Nebius</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO : actions Nebius</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO : action Nebius</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>Plus de 100 récompenses</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Frais de trading très bas</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Investissez à faible coût</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3M investisseurs satisfaits</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Plateforme primée</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Investir comporte un risque de perte. Ceci n'est pas un conseil en investissement.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Investissez dans l'action Nebius à faible coût avec DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Ouvrez un compte gratuit et accédez à 45+ marchés dans 30 pays.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Découvrez pourquoi 3M d'investisseurs utilisent notre plateforme primée.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>actions</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27597,7 +28508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -32978,6 +33889,280 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk akcje</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO: każdy może inwestować</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Zacznij inwestować z DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO: bardzo niskie opłaty</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO: siła finansowa</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Inwestuj w Sandisk z DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Akcje Sandisk</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Inwestuj w akcje Sandisk</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Inwestuj w akcję Sandisk</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO: akcje Sandisk</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO: akcja Sandisk</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>100+ nagród międzynarodowych</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Bardzo niskie opłaty</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Inwestuj przy niskich kosztach</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3 mln inwestorów ufa DEGIRO</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Nagradzana platforma</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Inwestowanie wiąże się z ryzykiem straty. To nie jest porada inwestycyjna.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Zacznij inwestować w akcje Sandisk przy niskich kosztach w DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Otwórz darmowe konto i zyskaj dostęp do 45+ rynków w 30 krajach.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Zobacz, dlaczego 3 mln inwestorów wybiera naszą nagradzaną platformę.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>akcje</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius akcje</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO: każdy może inwestować</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Zacznij inwestować z DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO: bardzo niskie opłaty</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO: siła finansowa</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Inwestuj w Nebius z DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Akcje Nebius</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Inwestuj w akcje Nebius</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Inwestuj w akcję Nebius</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO: akcje Nebius</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO: akcja Nebius</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>100+ nagród międzynarodowych</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Bardzo niskie opłaty</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Inwestuj przy niskich kosztach</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3 mln inwestorów ufa DEGIRO</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Nagradzana platforma</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Inwestowanie wiąże się z ryzykiem straty. To nie jest porada inwestycyjna.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Zacznij inwestować w akcje Nebius przy niskich kosztach w DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Otwórz darmowe konto i zyskaj dostęp do 45+ rynków w 30 krajach.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Zobacz, dlaczego 3 mln inwestorów wybiera naszą nagradzaną platformę.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>akcje</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -32989,7 +34174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -38370,6 +39555,280 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk ações</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO: todos podem investir</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Comece a investir com DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO: taxas muito baixas</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO: poder financeiro</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Invista em Sandisk - DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Ações da Sandisk</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Invista em ações da Sandisk</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Invista na ação da Sandisk</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO: ações da Sandisk</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO: ação da Sandisk</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>100+ prémios internacionais</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Comissões de negociação baixas</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Invista com custos baixos</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3M de investidores confiam</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Plataforma premiada</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Investir envolve risco de perda. Isto não é aconselhamento de investimento.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Comece a investir em ações da Sandisk com custos baixos na DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Abra a sua conta grátis e aceda a 45+ mercados em 30 países.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Descubra porque 3M investidores usam a nossa plataforma premiada.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>ações</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius ações</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO: todos podem investir</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Comece a investir com DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO: taxas muito baixas</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO: poder financeiro</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Invista em Nebius com a DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Ações da Nebius</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Invista em ações da Nebius</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Invista na ação da Nebius</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO: ações da Nebius</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO: ação da Nebius</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>100+ prémios internacionais</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Comissões de negociação baixas</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Invista com custos baixos</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3M de investidores confiam</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Plataforma premiada</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Investir envolve risco de perda. Isto não é aconselhamento de investimento.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Comece a investir em ações da Nebius com custos baixos na DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Abra a sua conta grátis e aceda a 45+ mercados em 30 países.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Descubra porque 3M investidores usam a nossa plataforma premiada.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>ações</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -38381,7 +39840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB39"/>
+  <dimension ref="A1:AB41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -43762,6 +45221,280 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Sandisk</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Sandisk azioni</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>DEGIRO: investire è per tutti</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Inizia a investire con DEGIRO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>DEGIRO: commissioni basse</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>DEGIRO: potere finanziario</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Investi in Sandisk con DEGIRO</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Azioni Sandisk</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>Investi in azioni Sandisk</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Investi nell'azione Sandisk</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>DEGIRO: azioni Sandisk</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>DEGIRO: azione Sandisk</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>100+ premi internazionali</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Commissioni di trading basse</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>Investi con costi bassi</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3M di investitori si fidano</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>Piattaforma pluripremiata</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>Investire comporta un rischio di perdita. Non è una consulenza di investimento.</t>
+        </is>
+      </c>
+      <c r="W40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>Inizia a investire in azioni Sandisk con costi bassi su DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr">
+        <is>
+          <t>Apri un conto gratuito e accedi a 45+ mercati in 30 paesi.</t>
+        </is>
+      </c>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>Scopri perché 3M di investitori scelgono la nostra piattaforma premiata.</t>
+        </is>
+      </c>
+      <c r="AA40" t="inlineStr">
+        <is>
+          <t>azioni</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>sandisk</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Nebius</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Nebius azioni</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NBIS</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.degiro.nl/lp/beleggen</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>DEGIRO: investire è per tutti</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Inizia a investire con DEGIRO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>DEGIRO: commissioni basse</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>DEGIRO: potere finanziario</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Investi in Nebius con DEGIRO</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Azioni Nebius</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Investi in azioni Nebius</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Investi nell'azione Nebius</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>DEGIRO: azioni Nebius</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>DEGIRO: azione Nebius</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>100+ premi internazionali</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Commissioni di trading basse</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>Investi con costi bassi</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>3M di investitori si fidano</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Piattaforma pluripremiata</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>Investire comporta un rischio di perdita. Non è una consulenza di investimento.</t>
+        </is>
+      </c>
+      <c r="W41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>Inizia a investire in azioni Nebius con costi bassi su DEGIRO.</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr">
+        <is>
+          <t>Apri un conto gratuito e accedi a 45+ mercati in 30 paesi.</t>
+        </is>
+      </c>
+      <c r="Z41" t="inlineStr">
+        <is>
+          <t>Scopri perché 3M di investitori scelgono la nostra piattaforma premiata.</t>
+        </is>
+      </c>
+      <c r="AA41" t="inlineStr">
+        <is>
+          <t>azioni</t>
+        </is>
+      </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>nebius</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>